<commit_message>
pm6V PCB finished.  Started last power board.
</commit_message>
<xml_diff>
--- a/Lasser_Driver_v5/pm6V/pm6V_BOM_digikey.xlsx
+++ b/Lasser_Driver_v5/pm6V/pm6V_BOM_digikey.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1054,7 +1054,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>IRF540NPBF</t>
+          <t>IRF540ZPBF</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>IRF540N</t>
+          <t>IRF540Z</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>N-MOSFET 100V 33A TO-220 (pos pre-reg pass)</t>
+          <t>N-MOSFET 100V 36A TO-220 (pos pre-reg pass; IRF540N replacement)</t>
         </is>
       </c>
     </row>
@@ -1605,6 +1605,146 @@
       <c r="G34" t="inlineStr">
         <is>
           <t>Shunt voltage ref adj 0.1% SOT-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>4</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>PMSSS 440 0050 PH</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>B&amp;F Fastener Supply</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>pm6V Q7-Q10 (TO-264 mount)</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>#4-40 x 1/2in screw</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Hardware (off-PCB)</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>SS pan-head machine screw #4-40 x 1/2in; TO-264 tab-&gt;657 heatsink (verify length vs boss, 3/8in alt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>4</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>FWSS 004</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>B&amp;F Fastener Supply</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>pm6V Q7-Q10 (TO-264 mount)</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>#4 flat washer</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Hardware (off-PCB)</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>SS #4 flat washer, nut side</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>4</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>INTLWZ 004</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>B&amp;F Fastener Supply</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>pm6V Q7-Q10 (TO-264 mount)</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>#4 int-tooth lock washer</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Hardware (off-PCB)</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Internal-tooth lock washer #4 (anti-loosen under nut, thermal cycling)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>4</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>HNZ 440</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>B&amp;F Fastener Supply</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>pm6V Q7-Q10 (TO-264 mount)</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>#4-40 hex nut</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Hardware (off-PCB)</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>#4-40 hex nut, zinc-plated steel</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Continued work on power booards.
</commit_message>
<xml_diff>
--- a/Lasser_Driver_v5/pm6V/pm6V_BOM_digikey.xlsx
+++ b/Lasser_Driver_v5/pm6V/pm6V_BOM_digikey.xlsx
@@ -1344,7 +1344,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>pm6V R24,R31</t>
+          <t>pm6V R25,R30</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1379,7 +1379,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>pm6V R25,R30</t>
+          <t>pm6V R24,R31</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">

</xml_diff>

<commit_message>
working on the digital pcb layout.  Mostly done.
</commit_message>
<xml_diff>
--- a/Lasser_Driver_v5/pm6V/pm6V_BOM_digikey.xlsx
+++ b/Lasser_Driver_v5/pm6V/pm6V_BOM_digikey.xlsx
@@ -824,7 +824,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Heatsink TO-264 vert 1in</t>
+          <t>Heatsink TO-264 [REPLACE-DOES NOT FIT]</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -834,7 +834,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Vert board-mount heatsink 657-series 1in ~10C/W for TO-264 pass Q7-Q10; fits 100x160 Eurocard</t>
+          <t>*** DOES NOT FIT TO-264 (channel ~16mm &lt; 20mm device) *** REPLACE with clip-on OMNI-UNI-PF-38 + OMNI-UC clip (Wakefield-Vette, DK 345-1600-ND / 345-1493-ND); clip mount leaves the 25.4mm pin holes unused. Trialing before permanent change. [orig: vert 657-series 1in for TO-264 pass Q7-Q10]</t>
         </is>
       </c>
     </row>

</xml_diff>